<commit_message>
feat: Enhance marketing API and frontend integration
- Updated marketing API to return detailed group stats and client contact results.
- Modified frontend API calls to handle new response structures, including success wrappers.
- Improved error handling and fallback mechanisms for user authentication.
- Added new marketing section in the sidebar for navigation.
- Enhanced import functionality with better file handling and user feedback.
- Fixed various issues related to client contact management and UI responsiveness.
- Added regression tests and updated documentation to reflect changes.
- Introduced new test import CSV for validation purposes.
</commit_message>
<xml_diff>
--- a/data/test_review_import.xlsx
+++ b/data/test_review_import.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Import" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,38 +431,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Universitas Indonesia</t>
+          <t>PT Test Indonesia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://ui.ac.id</t>
+          <t>pttest.co.id</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Institut Teknologi Bandung</t>
+          <t>CV Contoh</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://itb.ac.id</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Universitas Gadjah Mada</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://ugm.ac.id</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>